<commit_message>
Security hardening and stop tracking server/.env
Remove committed server/.env from the repo, ignore env files, add rate
limits, session rotation, OAuth state in Postgres, and security docs.
Rotate credentials locally; see docs/SECRET-ROTATION.md for history purge.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/PROMPT-LOG.xlsx
+++ b/docs/PROMPT-LOG.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="355">
   <si>
     <t>ID</t>
   </si>
@@ -977,6 +977,105 @@
   </si>
   <si>
     <t>See assistant response for full list</t>
+  </si>
+  <si>
+    <t>49</t>
+  </si>
+  <si>
+    <t>Contact widget copy email + snackbar</t>
+  </si>
+  <si>
+    <t>Email button should copy address and show feedback</t>
+  </si>
+  <si>
+    <t>Click copies email; button turns success green; snackbar Email copied to clipboard</t>
+  </si>
+  <si>
+    <t>Small UX polish</t>
+  </si>
+  <si>
+    <t>mailto still via social links list</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>Are you saving all prompts to designated file?</t>
+  </si>
+  <si>
+    <t>Confirm prompt logging to PROMPT-LOG</t>
+  </si>
+  <si>
+    <t>Explained AGENTS.md rule; docs/PROMPT-LOG.csv + npm run prompt-log:export → xlsx; not automatic without agent following rule</t>
+  </si>
+  <si>
+    <t>Meta accountability question</t>
+  </si>
+  <si>
+    <t>Could add CI check or pre-commit reminder for CSV row</t>
+  </si>
+  <si>
+    <t>This row confirms logging for this prompt</t>
+  </si>
+  <si>
+    <t>51</t>
+  </si>
+  <si>
+    <t>Security issues list and fix all possible</t>
+  </si>
+  <si>
+    <t>Create SECURITY.md and remediate audit findings</t>
+  </si>
+  <si>
+    <t>docs/SECURITY.md; .gitignore env; rate limit helmet origin check; approved privilege gate; session rotation; OAuth DB state; audit log; reset token hash POST validate; signed cookies; netlify/vercel headers</t>
+  </si>
+  <si>
+    <t>Comprehensive hardening pass</t>
+  </si>
+  <si>
+    <t>CAPTCHA and email verify left open; run npm run db:migrate after pull</t>
+  </si>
+  <si>
+    <t>Restart dev:server; users re-login after signed cookies</t>
+  </si>
+  <si>
+    <t>52</t>
+  </si>
+  <si>
+    <t>.env.example — remove or gitignore?</t>
+  </si>
+  <si>
+    <t>Clarify whether example env files should be tracked</t>
+  </si>
+  <si>
+    <t>Keep .env.example committed; gitignore already ignores .env but allows !.env.example templates</t>
+  </si>
+  <si>
+    <t>Good security hygiene question</t>
+  </si>
+  <si>
+    <t>Copy example → .env locally; never commit .env</t>
+  </si>
+  <si>
+    <t>53</t>
+  </si>
+  <si>
+    <t>Fix exposed secrets and clean up git</t>
+  </si>
+  <si>
+    <t>server/.env was on GitHub with real admin password</t>
+  </si>
+  <si>
+    <t>git rm --cached server/.env; rotated SESSION_SECRET + admin password locally; SECRET-ROTATION.md; commit security fixes; filter-repo instructions</t>
+  </si>
+  <si>
+    <t>User asked to fix and clean up</t>
+  </si>
+  <si>
+    <t>User must force-push after filter-repo</t>
+  </si>
+  <si>
+    <t>See docs/SECRET-ROTATION.md</t>
   </si>
 </sst>
 </file>
@@ -1413,7 +1512,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -2846,8 +2945,153 @@
         <v>321</v>
       </c>
     </row>
+    <row r="50" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A50" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I50" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="51" ht="45" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A51" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="F51" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="G51" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="H51" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="I51" s="3" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="52" ht="71" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A52" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="H52" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I52" s="2" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="53" ht="45" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A53" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>345</v>
+      </c>
+      <c r="F53" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="G53" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="H53" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="I53" s="3" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="54" ht="58" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A54" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="H54" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I54" s="2" t="s">
+        <v>354</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I49"/>
+  <autoFilter ref="A1:I54"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>